<commit_message>
Tres preguntas nuevas (Castilla y León 2026) y huecos de la lámina de ostomías rediseñados
- Preguntas 382-384: PEG y enterramiento del tope, melenas y HDA, control de la ascitis.
- Lámina: huecos con tarjetas redondeadas, sombra y halo animado en lugar de recuadros discontinuos;
  cubren por completo los rótulos originales y el estado de error es opaco.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcwkaUzTqRCcFM5qLcxoAV
</commit_message>
<xml_diff>
--- a/datos/digestivo/preguntas_digestivo.xlsx
+++ b/datos/digestivo/preguntas_digestivo.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA382"/>
+  <dimension ref="A1:AA385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -39331,6 +39331,285 @@
         </is>
       </c>
     </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Castilla y León · 2026</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Castilla y León</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>ostom</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>peg</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>Válida</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>En un paciente al que se le ha realizado una gastrostomía endoscópica percutánea sin extensión yeyunal, cuando el tracto de la gastrostomía se ha curado (después de aproximadamente una semana), para evitar el síndrome de enterramiento del tope interno de la gastrostomía, la sonda debe movilizarse de la siguiente manera:</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Girarse diariamente y moverse hacia dentro al menos una vez por semana (como mínimo 2 cm hasta 10 cm).</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Girarse cada 7 días y moverse hacia dentro al menos cada 15 días (como mínimo 2 cm hasta 10 cm).</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>No debe girarse, solo moverse hacia dentro y hacia fuera semanalmente.</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>No debe movilizarse bajo ningún concepto.</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="R383" t="inlineStr">
+        <is>
+          <t>Según la guía ESPEN de nutrición enteral domiciliaria, una vez curado el trayecto (hacia la semana), la PEG sin extensión yeyunal se gira a diario y se introduce al menos una vez por semana entre 2 y 10 cm. Así se evita que el tope interno quede incluido en la pared gástrica (síndrome de enterramiento o «buried bumper»).</t>
+        </is>
+      </c>
+      <c r="T383" t="inlineStr">
+        <is>
+          <t>Girar cada 7 días e introducir cada 15 es demasiado poco: el tope puede quedar enterrado entre movilizaciones.</t>
+        </is>
+      </c>
+      <c r="U383" t="inlineStr">
+        <is>
+          <t>Girar sí es necesario en la PEG sin extensión yeyunal; lo que no se gira es la que lleva extensión yeyunal (se desplazaría).</t>
+        </is>
+      </c>
+      <c r="V383" t="inlineStr">
+        <is>
+          <t>Inmovilizar la sonda es justo lo que favorece el enterramiento del tope interno.</t>
+        </is>
+      </c>
+      <c r="Z383" t="inlineStr">
+        <is>
+          <t>PEG curada (≈1 semana): girar a diario e introducir 2-10 cm al menos 1 vez por semana; con extensión yeyunal, no girar</t>
+        </is>
+      </c>
+      <c r="AA383" t="inlineStr">
+        <is>
+          <t>Redactado con IA (explicación, por qué no e idea clave): pendiente de validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Castilla y León · 2026</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Castilla y León</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>hemorragia</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>Válida</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>¿Cuál de los siguientes hallazgos orienta más hacia una hemorragia digestiva alta?:</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Rectorragia con sangre.</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Melenas.</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Dolor en fosa ilíaca derecha.</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>Diarrea.</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="R384" t="inlineStr">
+        <is>
+          <t>Las melenas (heces negras, brillantes, pegajosas y malolientes, «alquitranadas») indican sangre digerida y orientan a una hemorragia digestiva alta, por encima del ángulo de Treitz. La hematemesis es el otro signo típico de HDA.</t>
+        </is>
+      </c>
+      <c r="S384" t="inlineStr">
+        <is>
+          <t>La rectorragia (sangre roja por el ano) orienta a hemorragia digestiva baja; solo una HDA masiva y rápida puede producirla.</t>
+        </is>
+      </c>
+      <c r="U384" t="inlineStr">
+        <is>
+          <t>El dolor en FID orienta a apendicitis u otros procesos del ciego, no a sangrado alto.</t>
+        </is>
+      </c>
+      <c r="V384" t="inlineStr">
+        <is>
+          <t>La diarrea es inespecífica y no indica por sí misma hemorragia alta.</t>
+        </is>
+      </c>
+      <c r="Z384" t="inlineStr">
+        <is>
+          <t>Melenas o hematemesis = hemorragia digestiva alta (por encima del ángulo de Treitz); rectorragia = sobre todo baja</t>
+        </is>
+      </c>
+      <c r="AA384" t="inlineStr">
+        <is>
+          <t>Redactado con IA (explicación, por qué no e idea clave): pendiente de validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Castilla y León · 2026</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Castilla y León</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>higado</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>cirrosis</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>Válida</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>En un paciente con ascitis secundaria a cirrosis, la valoración diaria más útil para detectar cambios en la acumulación de líquido es:</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Tensión arterial.</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Frecuencia respiratoria.</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Peso corporal y perímetro abdominal.</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>Saturación de oxígeno.</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R385" t="inlineStr">
+        <is>
+          <t>La evolución de la ascitis se controla pesando al paciente a diario (misma hora, en ayunas, tras orinar, misma báscula y ropa) y midiendo el perímetro abdominal siempre en el mismo punto, a la altura del ombligo, marcado en la piel. Se completa con el balance hídrico.</t>
+        </is>
+      </c>
+      <c r="S385" t="inlineStr">
+        <is>
+          <t>La tensión arterial no cuantifica el líquido acumulado en el abdomen.</t>
+        </is>
+      </c>
+      <c r="T385" t="inlineStr">
+        <is>
+          <t>La frecuencia respiratoria solo cambia con ascitis a tensión y no mide la evolución día a día.</t>
+        </is>
+      </c>
+      <c r="V385" t="inlineStr">
+        <is>
+          <t>La saturación de oxígeno es un dato indirecto y tardío; no sirve para seguir la ascitis.</t>
+        </is>
+      </c>
+      <c r="Z385" t="inlineStr">
+        <is>
+          <t>Ascitis: peso diario (misma hora, báscula y ropa) y perímetro abdominal en el mismo punto (ombligo)</t>
+        </is>
+      </c>
+      <c r="AA385" t="inlineStr">
+        <is>
+          <t>Redactado con IA (explicación, por qué no e idea clave): pendiente de validar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:X377"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>